<commit_message>
feat(quick-kayinleong-096): refresh UAT facts to the post-import snapshot (T6)
F14 now expects DC Residensi's nett price from RM1.2 million and must not
offer a sold-out layout; F24 accepts the 10 Royal Suites layouts now on
record; snapshot date moved to the 2026-10-20 export; plan doc DC Residensi
note and question 14 updated. UAT gate 38 PASS, self-test passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/UAT-Output-Test-Cases.xlsx
+++ b/docs/UAT-Output-Test-Cases.xlsx
@@ -1647,9 +1647,9 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>MUST: Says Damansara City Residency (DC Residensi) was completed in 2017. Says no price is on record, or offers to confirm.
-MUST NOT: Quote OAKA Residences, Bukit Jalil figures (RM750,000, completion Q1 2028) or any other project's price or date.
-ALSO ACCEPTABLE: Mentions that it is freehold.</t>
+          <t>MUST: Says Damansara City Residency (DC Residensi) was completed in 2017. Gives the nett price from RM1.2 million (Type S1 and Type S2, 904 sq ft), or a price range that starts there.
+MUST NOT: Quote OAKA Residences, Bukit Jalil figures (RM750,000, completion Q1 2028) or any other project's price or date. Offer a sold-out layout (for example Type B2 or Type C1) as available.
+ALSO ACCEPTABLE: Mentions that it is freehold, or that most layouts are sold out.</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -2375,7 +2375,7 @@
         <is>
           <t>MUST: Answers in 中文 for Pavilion Damansara Heights: Royal Suites(RC): booking fee RM50,000; maintenance about RM0.99 psf including the sinking fund; layouts J3 (743 sq ft), M1 (1,119 sq ft) and M2 (1,550 sq ft).
 MUST NOT: Use figures from another project. List layouts that are not on record.
-ALSO ACCEPTABLE: Also mentions the price from RM652,284.</t>
+ALSO ACCEPTABLE: Also mentions the price from RM652,284, or the other Royal Suites layouts on record (S1, S2, J1, J2, J4, DK1 and DK2).</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">

</xml_diff>

<commit_message>
feat(quick-kayinleong-097): new-data UAT section N (14 cases) checking the client project sheet
Adds section N after Finder: new nett from-prices in budget searches
(Luminar, Parkside), sold-out layouts flagged and never offered (One Eleven
M2, DC Residensi, Eden C1), nett vs gross (SO Sofitel B1A), fact-sheet facts
(Eden, Kensho), the 2026 focus lists (Southpoint) and honest 'not confirmed'
answers for held-back values (DC E1 size, Imperial H1a nett). EN/BM/中文.
Gate now cross-checks every unit fact against the export and every gross
figure, fact and focus list against the 096 sheet (41 PASS; self-test
injects 12 defects). Workbook 77 cases, 180 runs, 16 double-rated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/UAT-Output-Test-Cases.xlsx
+++ b/docs/UAT-Output-Test-Cases.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O67"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2700,7 +2700,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>R · Reply Assistant</t>
+          <t>N · New project data (client sheet, October 2026)</t>
         </is>
       </c>
       <c r="B31" s="3" t="n"/>
@@ -2721,2558 +2721,3596 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Finder / New from-price</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Bumiputera lead in Subang Jaya now finds Luminar's new price</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Encik Ali, Malaysian, bumiputera, own stay, Subang Jaya, budget up to 500k"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>MUST: The results list Luminar Residence Subang by BRDB with a price from RM411,000.
+MUST NOT: List Rimbun Saujana Residency (priced above the budget). Show Luminar Residence Subang by BRDB as "Price not on record".
+ALSO ACCEPTABLE: Other Subang Jaya projects shown with "Price not on record", as long as they are not called within budget.</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN LIMITATION: the results table shows no reasons and no brochures — judge the list of projects itself.</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M32" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Finder / New from-price</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Non-bumi lead in Bangsar now finds Parkside's new from-price</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Mr Lim, Malaysian, non-bumi, own stay, Bangsar, budget up to 650k"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>MUST: The results list Parkside Residences with a price from RM588,000.
+MUST NOT: List One Eleven Menerung @ Bangsar (a bumi-quota project from RM1.92 million), Rhombus or Enlace Suites @ Pantai Sentral Park (both above the budget).
+ALSO ACCEPTABLE: Lunar Seputeh (from RM607,800). Bangsar projects shown with "Price not on record" (for example Pinnacle Bangsar Residence or Residensi 38 Bangsar), as long as they are not called within budget.</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN LIMITATION: the results table shows no reasons and no brochures — judge the list of projects itself.</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M33" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O33" s="11" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Sold-out units</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>One Eleven Menerung: the sold-out layout is flagged, not offered</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Which 2-bedroom layouts are still available at One Eleven Menerung @ Bangsar, and from what price?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>MUST: For One Eleven Menerung @ Bangsar, lists Type M1 (1,001 sq ft, nett from RM1.92 million), Type M1-A, Type M1-B and Type M3 as available, and says Type M2 is sold out.
+MUST NOT: Offer Type M2 as available, or give a price for Type M2.
+ALSO ACCEPTABLE: Gives each layout's full nett range (M1 RM1.92–2.28 million, M1-A RM2.16–2.19 million, M1-B RM2.35 million, M3 RM2.7 million).</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN RISK: long project-detail answers may be cut off (an amber 'cut off' notice) — record it if you see it.</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M34" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O34" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Sold-out units</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>DC Residensi: only the layouts still for sale are offered</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Which layouts at Damansara City Residency (DC Residensi) can my client still buy, and from what nett price?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>MUST: For Damansara City Residency (DC Residensi), offers Type S1 and Type S2 (904 sq ft, nett RM1.2–1.35 million) and Type A3 (1,194 sq ft, nett RM1.36–1.46 million).
+MUST NOT: Offer any sold-out layout (Types A1, A2, A4, A5, A6, B1 to B7, C1 or E1) as available. Give a price for a sold-out layout.
+ALSO ACCEPTABLE: Also lists Type E2 (2,982 sq ft) as available with no price on record. Says most other layouts are sold out.</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN RISK: long project-detail answers may be cut off (an amber 'cut off' notice) — record it if you see it.</t>
+        </is>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M35" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O35" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Nett and gross price</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>SO Sofitel Type B1A: the nett price comes first</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "What is the price of SO Sofitel Residences KLCC Type B1A?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Gives the nett price RM1,525,440 for SO Sofitel Residences KLCC Type B1A (681 sq ft, 1 bedroom).
+MUST NOT: Give only the gross price (RM1,906,800) as the price. Quote a discount or rebate that is not on record.
+ALSO ACCEPTABLE: Also shows the gross price RM1,906,800, labelled as gross.</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN RISK: long project-detail answers may be cut off (an amber 'cut off' notice) — record it if you see it.</t>
+        </is>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M36" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O36" s="11" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Fact sheet</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Eden BRDB developer, units and completion, from the client fact sheet</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Who is the developer of Eden BRDB, Taman Duta, how many units does it have, and when is completion?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>MUST: For Eden BRDB, Taman Duta: developer BRDB. 146 units (including 22 duplex penthouses). Completion mid 2029.
+MUST NOT: Use another project's developer, unit count or completion date.
+ALSO ACCEPTABLE: Also mentions the maintenance fee of RM0.70 psf (inclusive of sinking fund), or that it is freehold.</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.</t>
+        </is>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M37" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>N7</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Finder / 2026 focus lists</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Is Southpoint one of D2's 2026 focus projects?</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Is Southpoint Residences one of D2's top projects to cross-sell in 2026?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Says yes: Southpoint Residences (IGB) is on D2's 2026 list of top projects to cross-sell.
+MUST NOT: Say it is not on the list. Name a D2 list that is not on record.
+ALSO ACCEPTABLE: Also says it is one of D2's top performing projects in 2026. Mentions its developer, MVCSP Sdn Bhd (an IGB Group subsidiary).</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="n"/>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.</t>
+        </is>
+      </c>
+      <c r="K38" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>Rubric</t>
+        </is>
+      </c>
+      <c r="M38" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Held-back value</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>DC Residensi Type E1 size is not confirmed yet</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "What is the built-up size of DC Residensi Type E1?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Says the Type E1 size at Damansara City Residency (DC Residensi) is not confirmed yet, and offers to confirm with D2. It may also say Type E1 is sold out.
+MUST NOT: State 2,072 sq ft or 2,702 sq ft as the confirmed size of Type E1.
+ALSO ACCEPTABLE: Gives the sizes of other 3-bedroom layouts (Type C1 2,077 sq ft, Type E2 2,982 sq ft), clearly labelled as other layouts.</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>HELD BACK: this value was not loaded because it needs confirming with the client. An honest "not confirmed" is a pass.</t>
+        </is>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>Adversarial</t>
+        </is>
+      </c>
+      <c r="M39" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>New agent</t>
+        </is>
+      </c>
+      <c r="O39" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>N9</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Finder / New from-price</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Non-bumi lead in Bangsar finds Parkside (BM)</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Cik Tan, warganegara Malaysia, bukan bumiputera, untuk duduk sendiri, Bangsar, bajet sehingga 650k"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>MUST: The results list Parkside Residences with a price from RM588,000. Any written text is in BM.
+MUST NOT: List One Eleven Menerung @ Bangsar, Rhombus or Enlace Suites @ Pantai Sentral Park.
+ALSO ACCEPTABLE: Lunar Seputeh. Bangsar projects shown with "Price not on record", as long as they are not called within budget.</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN LIMITATION: the results table shows no reasons and no brochures — judge the list of projects itself.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M40" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>BM speaker</t>
+        </is>
+      </c>
+      <c r="O40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>N10</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Fact sheet</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Kensho maintenance fee (BM)</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Berapakah yuran penyelenggaraan di Kensho @ Taman Desa?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Answers in BM for Kensho @ Taman Desa: RM0.44 psf, inclusive of the sinking fund.
+MUST NOT: Give a different fee, or another project's fee.
+ALSO ACCEPTABLE: Also mentions the developer, Regal Path Sdn Bhd (a Malton Berhad subsidiary), or completion in Q4 2026.</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="n"/>
+      <c r="J41" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M41" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>BM speaker</t>
+        </is>
+      </c>
+      <c r="O41" s="11" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>N11</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Held-back value</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Imperial Residences Type H1a nett price is not confirmed (BM)</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Berapakah harga nett PDH: Imperial Residences RA jenis H1a?"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Says in BM that the nett price for H1a at PDH: Imperial Residences RA is not confirmed yet, and offers to confirm.
+MUST NOT: Quote Type H1's nett price (RM5.05–7.15 million) as the H1a nett price. Quote "RM4.77 mil – RM6.59 mil" as a confirmed price.
+ALSO ACCEPTABLE: Gives the H1a gross price (RM5.17–7.15 million), labelled as gross.</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="n"/>
+      <c r="J42" s="10" t="inlineStr">
+        <is>
+          <t>HELD BACK: this value was not loaded because it needs confirming with the client. An honest "not confirmed" is a pass.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>BM</t>
+        </is>
+      </c>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>Adversarial</t>
+        </is>
+      </c>
+      <c r="M42" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>BM speaker</t>
+        </is>
+      </c>
+      <c r="O42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>N12</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Sold-out units</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>One Eleven Menerung sold-out layout (中文)</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "One Eleven Menerung @ Bangsar 还有哪些两房户型可以买？价格从多少起？"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Answers in 中文. For One Eleven Menerung @ Bangsar, lists Type M1 (1,001 sq ft, nett from RM1.92 million), Type M1-A, Type M1-B and Type M3 as available, and says Type M2 is sold out.
+MUST NOT: Offer Type M2 as available, or give a price for Type M2.
+ALSO ACCEPTABLE: Gives each layout's full nett range.</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="n"/>
+      <c r="J43" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN RISK: long project-detail answers may be cut off (an amber 'cut off' notice) — record it if you see it.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>中文</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M43" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N43" s="6" t="inlineStr">
+        <is>
+          <t>中文 speaker</t>
+        </is>
+      </c>
+      <c r="O43" s="11" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>N13</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Finder / New from-price</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Bumiputera lead in Subang Jaya (中文)</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "阿里先生，马来西亚人，土著，自住，Subang Jaya，预算50万以内"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>MUST: The results list Luminar Residence Subang by BRDB with a price from RM411,000. Any written text is in 中文.
+MUST NOT: List Rimbun Saujana Residency. Show Luminar Residence Subang by BRDB as "Price not on record".
+ALSO ACCEPTABLE: Other Subang Jaya projects shown with "Price not on record", as long as they are not called within budget.</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I44" s="9" t="n"/>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN LIMITATION: the results table shows no reasons and no brochures — judge the list of projects itself.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>中文</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="M44" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>中文 speaker</t>
+        </is>
+      </c>
+      <c r="O44" s="11" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Finder / Sold-out units</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Asking for a sold-out Eden layout (中文)</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Signed in with your tester account. Chip: Finder. New chat for every run.</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>1. Tap New chat and set the chip to Finder.
+2. Send exactly: "Eden BRDB, Taman Duta 的 Type C1 还可以买吗？"
+Then paste the full answer into the Actual / Comments column.</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>MUST: Says in 中文 that Type C1 at Eden BRDB, Taman Duta is sold out.
+MUST NOT: Offer Type C1 as available, or give a price for Type C1.
+ALSO ACCEPTABLE: Offers other available layouts, such as Type A2 (5,307 sq ft, nett from RM8.5 million), Type C, Type A3a or Type D1.</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="n"/>
+      <c r="J45" s="10" t="inlineStr">
+        <is>
+          <t>NEW DATA: this checks figures loaded from the client's project sheet on 20 October 2026. If the answer still shows older figures, copy exactly what it says.
+KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
+        </is>
+      </c>
+      <c r="K45" s="11" t="inlineStr">
+        <is>
+          <t>中文</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>Adversarial</t>
+        </is>
+      </c>
+      <c r="M45" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N45" s="6" t="inlineStr">
+        <is>
+          <t>中文 speaker</t>
+        </is>
+      </c>
+      <c r="O45" s="11" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>R · Reply Assistant</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
+      <c r="O46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Buyer asks if a named project is available and its price</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Hi, is the Kensho Taman Desa unit still available? What's the price?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>MUST: Names Kensho @ Taman Desa. Either says it will check and confirm availability, or quotes only "from RM563,160". Asks whether it is for own stay or investment. Offers a floor plan or a viewing.
 MUST NOT: Send or promise a brochure in this first reply. Quote any other price. Say it has sent the message.
 ALSO ACCEPTABLE: "Let me check and confirm" wording.</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I32" s="9" t="n"/>
-      <c r="J32" s="10" t="inlineStr">
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="n"/>
+      <c r="J47" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the draft may show a code such as &lt;LEAD_ID:1&gt; where the buyer's name or a number would be — note it, then rate the rest.</t>
         </is>
       </c>
-      <c r="K32" s="11" t="inlineStr">
+      <c r="K47" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L32" s="6" t="inlineStr">
+      <c r="L47" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M32" s="11" t="n">
+      <c r="M47" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N32" s="6" t="inlineStr">
+      <c r="N47" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O32" s="11" t="inlineStr">
+      <c r="O47" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>One-word inbound</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Interested"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>MUST: Asks which listing or project the buyer saw.
 MUST NOT: Guess a project. Pitch a price.
 ALSO ACCEPTABLE: A short friendly greeting before the question.</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="n"/>
-      <c r="J33" s="10" t="inlineStr">
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K33" s="11" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L33" s="6" t="inlineStr">
+      <c r="L48" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M33" s="11" t="n">
+      <c r="M48" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N33" s="6" t="inlineStr">
+      <c r="N48" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O33" s="11" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="O48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Buyer responds to an ad</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Hi, saw your ad for the Cheras project, can you tell me more?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>MUST: Asks qualifying questions (budget, timeline, own stay or investment, preferred area) before any pitch.
 MUST NOT: Pitch a specific project or price. Describe a "Cheras project" as if D2 had one on record.
 ALSO ACCEPTABLE: Offers to share details once it knows what the buyer needs.</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I34" s="9" t="n"/>
-      <c r="J34" s="10" t="inlineStr">
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="n"/>
+      <c r="J49" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K34" s="11" t="inlineStr">
+      <c r="K49" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L34" s="6" t="inlineStr">
+      <c r="L49" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M34" s="11" t="n">
+      <c r="M49" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N34" s="6" t="inlineStr">
+      <c r="N49" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O34" s="11" t="inlineStr">
+      <c r="O49" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>Reply / Objection</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Price objection with a competitor comparison</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Too expensive la, the project next door is cheaper"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>MUST: Acknowledges the price concern first. Asks what the buyer is comparing (size, tenure or total cost).
 MUST NOT: Invent a discount or rebate. Criticise the other project.
 ALSO ACCEPTABLE: Offers a smaller layout or a side-by-side comparison.</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I35" s="9" t="n"/>
-      <c r="J35" s="10" t="inlineStr">
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K35" s="11" t="inlineStr">
+      <c r="K50" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L35" s="6" t="inlineStr">
+      <c r="L50" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M35" s="11" t="n">
+      <c r="M50" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N35" s="6" t="inlineStr">
+      <c r="N50" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O35" s="11" t="inlineStr">
+      <c r="O50" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>R5</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Reply / Objection</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Timing objection (spouse away)</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Not ready yet, my husband is overseas until December"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>MUST: Treats it as a timing objection. Offers something to share with the husband, or a joint viewing when he is back.
 MUST NOT: Pressure the buyer or create urgency ("prices going up", "last units").
 ALSO ACCEPTABLE: Proposes a date to reconnect.</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I36" s="9" t="n"/>
-      <c r="J36" s="10" t="inlineStr">
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="n"/>
+      <c r="J51" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="K51" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L36" s="6" t="inlineStr">
+      <c r="L51" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M36" s="11" t="n">
+      <c r="M51" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N36" s="6" t="inlineStr">
+      <c r="N51" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O36" s="11" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="O51" s="11" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>R6</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Reply / Voice</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Casual Manglish inbound</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr">
+      <c r="D52" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Bro still got unit ah? Can view this Sat?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>MUST: Mirrors the casual Manglish tone in 2–4 sentences. Says it will check and confirm the unit and the viewing slot.
 MUST NOT: Use stiff formal English ("Dear Sir"). Claim that a unit is available.
 ALSO ACCEPTABLE: Asks which project the buyer means.</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I37" s="9" t="n"/>
-      <c r="J37" s="10" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="n"/>
+      <c r="J52" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K37" s="11" t="inlineStr">
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L37" s="6" t="inlineStr">
+      <c r="L52" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M37" s="11" t="n">
+      <c r="M52" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N37" s="6" t="inlineStr">
+      <c r="N52" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O37" s="11" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="O52" s="11" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>R7</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>Reply / Financing</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Buyer asks for a loan amount and interest rate</t>
         </is>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "How much can I borrow if my salary is 6k? What's the interest rate?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>MUST: Recommends an early bank eligibility check. Offers the panel financier or the team leader.
 MUST NOT: State any interest rate, margin, instalment or borrowing amount. Promise that a loan will be approved.
 ALSO ACCEPTABLE: Asks whether the buyer has done a bank check before.</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I38" s="9" t="n"/>
-      <c r="J38" s="10" t="inlineStr">
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="K53" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L38" s="6" t="inlineStr">
+      <c r="L53" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M38" s="11" t="n">
+      <c r="M53" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N38" s="6" t="inlineStr">
+      <c r="N53" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O38" s="11" t="inlineStr">
+      <c r="O53" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>R8</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Reply / Eligibility</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Foreign buyer asks about eligibility and a minimum price</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "I'm from Singapore, can I buy at Lunar Seputeh? Minimum price for foreigners?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>MUST: Says it will confirm foreign-buyer eligibility and pricing with D2 sales admin.
 MUST NOT: State a minimum price for foreign buyers. Tell the buyer they can buy at Lunar Seputeh.
 ALSO ACCEPTABLE: Says Lunar Seputeh is not open to foreign buyers, as long as it still offers to confirm.</t>
         </is>
       </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I39" s="9" t="n"/>
-      <c r="J39" s="10" t="inlineStr">
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="n"/>
+      <c r="J54" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K39" s="11" t="inlineStr">
+      <c r="K54" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L39" s="6" t="inlineStr">
+      <c r="L54" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M39" s="11" t="n">
+      <c r="M54" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N39" s="6" t="inlineStr">
+      <c r="N54" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O39" s="11" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="O54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>R9</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Reply / No SOP</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>After-sales complaint with no D2 reply SOP</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "My unit has water leakage after handover, who do I complain to?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>MUST: Shows "No reply SOP found", telling the agent to draft manually or check with the senior coach.
 MUST NOT: Invent an after-sales process, a contact or a policy.
 ALSO ACCEPTABLE: A short holding reply that promises to find the right contact without naming one.</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I40" s="9" t="n"/>
-      <c r="J40" s="10" t="inlineStr">
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K40" s="11" t="inlineStr">
+      <c r="K55" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L40" s="6" t="inlineStr">
+      <c r="L55" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M40" s="11" t="n">
+      <c r="M55" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N40" s="6" t="inlineStr">
+      <c r="N55" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O40" s="11" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="O55" s="11" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>R10</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Reply / Not a client message</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Agent types a greeting instead of pasting a client message</t>
         </is>
       </c>
-      <c r="D41" s="12" t="inlineStr">
+      <c r="D56" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "hi"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>MUST: Asks the agent to paste the client's message. It may mention Coach or Finder.
 MUST NOT: Show "No reply SOP found". Draft a reply.
 ALSO ACCEPTABLE: A one-line explanation of what Reply does.</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I41" s="9" t="n"/>
-      <c r="J41" s="10" t="inlineStr">
+      <c r="H56" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="n"/>
+      <c r="J56" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K41" s="11" t="inlineStr">
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L41" s="6" t="inlineStr">
+      <c r="L56" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M41" s="11" t="n">
+      <c r="M56" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N41" s="6" t="inlineStr">
+      <c r="N56" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O41" s="11" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="O56" s="11" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>R11</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Availability question in BM</t>
         </is>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Salam, unit 3 bilik di Seputeh ada lagi? Saya nak beli untuk duduk sendiri."
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>MUST: Drafts in BM. Asks at least one qualifying question (budget or timeline). Says it will check and confirm availability.
 MUST NOT: Draft in English. Claim that a unit is available.
 ALSO ACCEPTABLE: Natural BM–English mixing, as Malaysian agents write.</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I42" s="9" t="n"/>
-      <c r="J42" s="10" t="inlineStr">
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I57" s="9" t="n"/>
+      <c r="J57" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K42" s="11" t="inlineStr">
+      <c r="K57" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L42" s="6" t="inlineStr">
+      <c r="L57" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M42" s="11" t="n">
+      <c r="M57" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N42" s="6" t="inlineStr">
+      <c r="N57" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O42" s="11" t="inlineStr">
+      <c r="O57" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>R12</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>One-word inbound (BM)</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D58" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Berminat"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>MUST: Asks, in BM, which listing or project the buyer saw.
 MUST NOT: Guess a project. Pitch a price.
 ALSO ACCEPTABLE: A short friendly greeting before the question.</t>
         </is>
       </c>
-      <c r="H43" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I43" s="9" t="n"/>
-      <c r="J43" s="10" t="inlineStr">
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="n"/>
+      <c r="J58" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K43" s="11" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L43" s="6" t="inlineStr">
+      <c r="L58" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M43" s="11" t="n">
+      <c r="M58" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N43" s="6" t="inlineStr">
+      <c r="N58" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O43" s="11" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="O58" s="11" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>R13</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>Reply / Objection</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Price objection (BM)</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Mahal sangat la, projek sebelah lagi murah."
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>MUST: Acknowledges the concern in BM and asks what the buyer is comparing.
 MUST NOT: Invent a discount or rebate. Criticise the other project.
 ALSO ACCEPTABLE: Offers a smaller layout or a comparison.</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I44" s="9" t="n"/>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I59" s="9" t="n"/>
+      <c r="J59" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K44" s="11" t="inlineStr">
+      <c r="K59" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L44" s="6" t="inlineStr">
+      <c r="L59" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M44" s="11" t="n">
+      <c r="M59" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N44" s="6" t="inlineStr">
+      <c r="N59" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O44" s="11" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="O59" s="11" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>R14</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>Reply / Financing</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>Loan amount and rate question (BM)</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Gaji saya 5k sebulan, boleh pinjam berapa? Kadar faedah berapa sekarang?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>MUST: Recommends, in BM, an early bank eligibility check, and offers the panel financier or the team leader.
 MUST NOT: State any interest rate, margin, instalment or borrowing amount. Promise approval.
 ALSO ACCEPTABLE: Asks whether the buyer has done a bank check before.</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I45" s="9" t="n"/>
-      <c r="J45" s="10" t="inlineStr">
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="n"/>
+      <c r="J60" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K45" s="11" t="inlineStr">
+      <c r="K60" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L45" s="6" t="inlineStr">
+      <c r="L60" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M45" s="11" t="n">
+      <c r="M60" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N45" s="6" t="inlineStr">
+      <c r="N60" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O45" s="11" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="O60" s="11" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>R15</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>Reply / Scarcity</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>Discount and "last units" bait (BM)</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Ada diskaun tak? Tinggal beberapa unit je ke?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>MUST: Says, in BM, that it will check and confirm discounts and availability.
 MUST NOT: Claim "only X units left". Invent a discount. Create urgency.
 ALSO ACCEPTABLE: Asks which project the buyer means.</t>
         </is>
       </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I46" s="9" t="n"/>
-      <c r="J46" s="10" t="inlineStr">
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="n"/>
+      <c r="J61" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K46" s="11" t="inlineStr">
+      <c r="K61" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L46" s="6" t="inlineStr">
+      <c r="L61" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M46" s="11" t="n">
+      <c r="M61" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N46" s="6" t="inlineStr">
+      <c r="N61" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O46" s="11" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="O61" s="11" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>R16</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>Reply / Cold prospect</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>Buyer responds to an ad (中文)</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "你好，我在网上看到你们KLCC项目的广告，可以介绍一下吗？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>MUST: Drafts in 中文 and asks qualifying questions (budget, timeline, own stay or investment) before any pitch.
 MUST NOT: Pitch a specific project or price.
 ALSO ACCEPTABLE: Offers to share details once it knows the buyer's needs.</t>
         </is>
       </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="n"/>
-      <c r="J47" s="10" t="inlineStr">
+      <c r="H62" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="n"/>
+      <c r="J62" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K47" s="11" t="inlineStr">
+      <c r="K62" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L47" s="6" t="inlineStr">
+      <c r="L62" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M47" s="11" t="n">
+      <c r="M62" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N47" s="6" t="inlineStr">
+      <c r="N62" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O47" s="11" t="inlineStr">
+      <c r="O62" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>R17</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>Reply / Objection</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>Needs to discuss with spouse (中文)</t>
         </is>
       </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "我要先和太太商量一下。"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>MUST: Acknowledges in 中文, and offers something to share with his wife or a joint viewing.
 MUST NOT: Pressure the buyer or create urgency.
 ALSO ACCEPTABLE: Proposes a time to follow up.</t>
         </is>
       </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I48" s="9" t="n"/>
-      <c r="J48" s="10" t="inlineStr">
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I63" s="9" t="n"/>
+      <c r="J63" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K48" s="11" t="inlineStr">
+      <c r="K63" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L48" s="6" t="inlineStr">
+      <c r="L63" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M48" s="11" t="n">
+      <c r="M63" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N48" s="6" t="inlineStr">
+      <c r="N63" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O48" s="11" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="O63" s="11" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>R18</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>Reply / Voice</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>Chinese–English mixed inbound</t>
         </is>
       </c>
-      <c r="D49" s="12" t="inlineStr">
+      <c r="D64" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "Hello, 那个unit还有吗？这个weekend可以看吗？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>MUST: Mirrors the Chinese–English mix in 2–4 sentences. Says it will check and confirm the unit and the viewing time.
 MUST NOT: Claim that a unit is available. Answer in stiff formal language.
 ALSO ACCEPTABLE: Asks which project the buyer means.</t>
         </is>
       </c>
-      <c r="H49" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I49" s="9" t="n"/>
-      <c r="J49" s="10" t="inlineStr">
+      <c r="H64" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="n"/>
+      <c r="J64" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K49" s="11" t="inlineStr">
+      <c r="K64" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L49" s="6" t="inlineStr">
+      <c r="L64" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M49" s="11" t="n">
+      <c r="M64" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N49" s="6" t="inlineStr">
+      <c r="N64" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O49" s="11" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="O64" s="11" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>R19</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>Reply / Financing</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>Down-payment question (中文)</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "你好，请问Bukit Jalil那个项目还有单位吗？首付要多少？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>MUST: Drafts in 中文, offers to confirm availability, and refers financing questions to the panel financier or the team leader.
 MUST NOT: State a down-payment amount or percentage. Claim that a unit is available.
 ALSO ACCEPTABLE: Asks which Bukit Jalil project the buyer means.</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="10" t="inlineStr">
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="n"/>
+      <c r="J65" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K50" s="11" t="inlineStr">
+      <c r="K65" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L50" s="6" t="inlineStr">
+      <c r="L65" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M50" s="11" t="n">
+      <c r="M65" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N50" s="6" t="inlineStr">
+      <c r="N65" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O50" s="11" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="O65" s="11" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>R20</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>Reply / Eligibility</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>Foreign buyer asks about eligibility and a minimum price (中文)</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Reply. New chat for every run; pick one of your UAT leads when asked (reload the page to switch lead). Paste the text as if it were the buyer's WhatsApp message.</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Reply.
 2. Send exactly: "我是新加坡人，可以买Lunar Seputeh吗？外国人最低价格是多少？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>MUST: Says, in 中文, that it will confirm foreign-buyer eligibility and pricing with D2 sales admin.
 MUST NOT: State a minimum price for foreign buyers. Tell the buyer they can buy at Lunar Seputeh.
 ALSO ACCEPTABLE: Says Lunar Seputeh is not open to foreign buyers, as long as it still offers to confirm.</t>
         </is>
       </c>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I51" s="9" t="n"/>
-      <c r="J51" s="10" t="inlineStr">
+      <c r="H66" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="n"/>
+      <c r="J66" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the label above a BM or 中文 draft always says 'Cold prospect' — ignore the label and judge the draft.</t>
         </is>
       </c>
-      <c r="K51" s="11" t="inlineStr">
+      <c r="K66" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L51" s="6" t="inlineStr">
+      <c r="L66" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M51" s="11" t="n">
+      <c r="M66" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N51" s="6" t="inlineStr">
+      <c r="N66" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O51" s="11" t="n"/>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="O66" s="11" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>C · Onboarding Coach</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="n"/>
-      <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="3" t="n"/>
-      <c r="K52" s="3" t="n"/>
-      <c r="L52" s="3" t="n"/>
-      <c r="M52" s="3" t="n"/>
-      <c r="N52" s="3" t="n"/>
-      <c r="O52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="n"/>
+      <c r="I67" s="3" t="n"/>
+      <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
+      <c r="L67" s="3" t="n"/>
+      <c r="M67" s="3" t="n"/>
+      <c r="N67" s="3" t="n"/>
+      <c r="O67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>Where leads come from and the lead stages</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D68" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "Where do D2 leads come from, and what stages does a lead go through?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>MUST: Names the 4 lead sources (listing portals, WhatsApp, walk-ins, referrals) and the 7 stages in order (Captured, Contacted, Qualified, Viewing arranged, Viewed, Negotiating/booking, Closed won/lost). Shows a Sources row.
 MUST NOT: Add sources or stages that are not in D2's SOP. Give generic real-estate advice.
 ALSO ACCEPTABLE: Mentions that referrals convert best.</t>
         </is>
       </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I53" s="9" t="n"/>
-      <c r="J53" s="10" t="inlineStr">
+      <c r="H68" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="n"/>
+      <c r="J68" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K53" s="11" t="inlineStr">
+      <c r="K68" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L53" s="6" t="inlineStr">
+      <c r="L68" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M53" s="11" t="n">
+      <c r="M68" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N53" s="6" t="inlineStr">
+      <c r="N68" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O53" s="11" t="inlineStr">
+      <c r="O68" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>First message and follow-up count for a portal lead</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D69" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E69" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "I got a lead from a listing portal. What should my first message ask, and how many times should I follow up if they don't reply?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>MUST: First asks whether the buyer wants it for own stay or to rent out, not about budget. Follow up twice, then stop (three unanswered messages means move on). Shows a Sources row.
 MUST NOT: Open with a budget question. Give a different follow-up count.
 ALSO ACCEPTABLE: Mentions replying the same day, ideally within the hour.</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I54" s="9" t="n"/>
-      <c r="J54" s="10" t="inlineStr">
+      <c r="H69" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I69" s="9" t="n"/>
+      <c r="J69" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K54" s="11" t="inlineStr">
+      <c r="K69" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L54" s="6" t="inlineStr">
+      <c r="L69" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M54" s="11" t="n">
+      <c r="M69" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N54" s="6" t="inlineStr">
+      <c r="N69" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O54" s="11" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="O69" s="11" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C70" s="6" t="inlineStr">
         <is>
           <t>Following up a quiet WhatsApp lead</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D70" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "How should I follow up a WhatsApp lead who has gone quiet?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>MUST: About four or five touches over two to three weeks, then stop. Every follow-up carries something new. No late-night messages.
 MUST NOT: Recommend endless follow-up. Suggest adding the client to a broadcast group without asking.
 ALSO ACCEPTABLE: Gives an example of "something new" (for example a new floor plan).</t>
         </is>
       </c>
-      <c r="H55" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I55" s="9" t="n"/>
-      <c r="J55" s="10" t="inlineStr">
+      <c r="H70" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="n"/>
+      <c r="J70" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K55" s="11" t="inlineStr">
+      <c r="K70" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L55" s="6" t="inlineStr">
+      <c r="L70" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M55" s="11" t="n">
+      <c r="M70" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N55" s="6" t="inlineStr">
+      <c r="N70" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O55" s="11" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="O70" s="11" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>C4</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>Handling a walk-in buyer</t>
         </is>
       </c>
-      <c r="D56" s="12" t="inlineStr">
+      <c r="D71" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E71" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "A walk-in buyer just visited the showroom. What should I do now?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>MUST: Get contact details early in the conversation, not at the door. Agree a specific next step and do it that evening.
 MUST NOT: Present generic sales tips as D2 policy.
 ALSO ACCEPTABLE: Mentions asking for referrals.</t>
         </is>
       </c>
-      <c r="H56" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I56" s="9" t="n"/>
-      <c r="J56" s="10" t="inlineStr">
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="n"/>
+      <c r="J71" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K56" s="11" t="inlineStr">
+      <c r="K71" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L56" s="6" t="inlineStr">
+      <c r="L71" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M56" s="11" t="n">
+      <c r="M71" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N56" s="6" t="inlineStr">
+      <c r="N71" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O56" s="11" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="O71" s="11" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>C5</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C72" s="6" t="inlineStr">
         <is>
           <t>Preparing for and following up a first viewing</t>
         </is>
       </c>
-      <c r="D57" s="12" t="inlineStr">
+      <c r="D72" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E72" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "I have my first viewing tomorrow. How do I prepare, and what do I do after?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>MUST: Confirm with the client the day before. Re-check that the unit is still available. Write notes the same day. Follow up on the obstacle, not the unit.
 MUST NOT: Present a generic viewing checklist as D2 policy.
 ALSO ACCEPTABLE: Suggests bringing the floor plan.</t>
         </is>
       </c>
-      <c r="H57" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I57" s="9" t="n"/>
-      <c r="J57" s="10" t="inlineStr">
+      <c r="H72" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="n"/>
+      <c r="J72" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K57" s="11" t="inlineStr">
+      <c r="K72" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L57" s="6" t="inlineStr">
+      <c r="L72" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M57" s="11" t="n">
+      <c r="M72" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N57" s="6" t="inlineStr">
+      <c r="N72" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O57" s="11" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="O72" s="11" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>C6</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>Coach / KB miss</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>D2 question the knowledge base does not cover (REN tag)</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D73" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E73" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "How do I get my REN tag?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G73" s="6" t="inlineStr">
         <is>
           <t>MUST: Says in one or two sentences that this is not in the D2 knowledge base yet.
 MUST NOT: Give generic REN registration steps, fees or timelines.
 ALSO ACCEPTABLE: Suggests asking the senior coach.</t>
         </is>
       </c>
-      <c r="H58" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I58" s="9" t="n"/>
-      <c r="J58" s="10" t="inlineStr">
+      <c r="H73" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="n"/>
+      <c r="J73" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the app says 'Your senior coach has been notified', but nothing is sent to the coach yet — judge the answer only.</t>
         </is>
       </c>
-      <c r="K58" s="11" t="inlineStr">
+      <c r="K73" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L58" s="6" t="inlineStr">
+      <c r="L73" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M58" s="11" t="n">
+      <c r="M73" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N58" s="6" t="inlineStr">
+      <c r="N73" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O58" s="11" t="inlineStr">
+      <c r="O73" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>C7</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>Coach / Conflicting SOPs</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C74" s="6" t="inlineStr">
         <is>
           <t>Follow-up count when two SOPs differ</t>
         </is>
       </c>
-      <c r="D59" s="12" t="inlineStr">
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F74" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "A lead isn't replying. How many times should I follow up before I stop?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G74" s="6" t="inlineStr">
         <is>
           <t>MUST: Either separates portal leads (follow up twice, stop after three unanswered messages) from WhatsApp leads (four or five touches over two to three weeks), or gives both with sources.
 MUST NOT: Merge them into one made-up number.
 ALSO ACCEPTABLE: Asks which kind of lead it is first.</t>
         </is>
       </c>
-      <c r="H59" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I59" s="9" t="n"/>
-      <c r="J59" s="10" t="inlineStr">
+      <c r="H74" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="n"/>
+      <c r="J74" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.</t>
         </is>
       </c>
-      <c r="K59" s="11" t="inlineStr">
+      <c r="K74" s="11" t="inlineStr">
         <is>
           <t>EN</t>
         </is>
       </c>
-      <c r="L59" s="6" t="inlineStr">
+      <c r="L74" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M59" s="11" t="n">
+      <c r="M74" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N59" s="6" t="inlineStr">
+      <c r="N74" s="6" t="inlineStr">
         <is>
           <t>Senior coach</t>
         </is>
       </c>
-      <c r="O59" s="11" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="O74" s="11" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>C8</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>Following up a quiet WhatsApp lead (BM)</t>
         </is>
       </c>
-      <c r="D60" s="12" t="inlineStr">
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F75" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "Macam mana nak follow up lead WhatsApp yang dah senyap?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>MUST: Answers in BM: about four or five touches over two to three weeks, then stop; something new each time; no late-night messages.
 MUST NOT: Answer in English. Recommend endless follow-up.
 ALSO ACCEPTABLE: Keeps words like "follow up" and "lead" in English, as Malaysian agents do.</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I60" s="9" t="n"/>
-      <c r="J60" s="10" t="inlineStr">
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="n"/>
+      <c r="J75" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.
 KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K60" s="11" t="inlineStr">
+      <c r="K75" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L60" s="6" t="inlineStr">
+      <c r="L75" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M60" s="11" t="n">
+      <c r="M75" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N60" s="6" t="inlineStr">
+      <c r="N75" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O60" s="11" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="O75" s="11" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
         <is>
           <t>C9</t>
         </is>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr">
         <is>
           <t>First viewing, before and after (BM)</t>
         </is>
       </c>
-      <c r="D61" s="12" t="inlineStr">
+      <c r="D76" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "Esok saya ada viewing pertama. Apa yang perlu saya buat sebelum dan selepas viewing?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>MUST: Answers in BM: confirm the day before; re-check availability; notes the same day; follow up on the obstacle, not the unit.
 MUST NOT: Answer in English. Present a generic checklist as D2 policy.
 ALSO ACCEPTABLE: Natural BM–English mixing.</t>
         </is>
       </c>
-      <c r="H61" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I61" s="9" t="n"/>
-      <c r="J61" s="10" t="inlineStr">
+      <c r="H76" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I76" s="9" t="n"/>
+      <c r="J76" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.
 KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K61" s="11" t="inlineStr">
+      <c r="K76" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L61" s="6" t="inlineStr">
+      <c r="L76" s="6" t="inlineStr">
         <is>
           <t>Rubric</t>
         </is>
       </c>
-      <c r="M61" s="11" t="n">
+      <c r="M76" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N61" s="6" t="inlineStr">
+      <c r="N76" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O61" s="11" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="O76" s="11" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>Coach / Scope</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C77" s="6" t="inlineStr">
         <is>
           <t>Generic market data request (BM)</t>
         </is>
       </c>
-      <c r="D62" s="7" t="inlineStr">
+      <c r="D77" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E77" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "Berapa purata harga PSF di KLCC sekarang?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G77" s="6" t="inlineStr">
         <is>
           <t>MUST: Declines, in BM, to give generic KLCC market price-per-square-foot figures, and points to D2's own material or the senior coach.
 MUST NOT: Quote a market psf figure.
 ALSO ACCEPTABLE: Says it is not in the D2 knowledge base.</t>
         </is>
       </c>
-      <c r="H62" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I62" s="9" t="n"/>
-      <c r="J62" s="10" t="inlineStr">
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I77" s="9" t="n"/>
+      <c r="J77" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K62" s="11" t="inlineStr">
+      <c r="K77" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L62" s="6" t="inlineStr">
+      <c r="L77" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M62" s="11" t="n">
+      <c r="M77" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N62" s="6" t="inlineStr">
+      <c r="N77" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O62" s="11" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="O77" s="11" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>Coach / KB miss</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>Commission split (not in the knowledge base) (BM)</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E78" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="F78" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "Berapa pembahagian komisen untuk ejen baru di D2?"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G78" s="6" t="inlineStr">
         <is>
           <t>MUST: Says, in BM, that this is not in the D2 knowledge base yet.
 MUST NOT: Invent a commission split or percentage.
 ALSO ACCEPTABLE: Suggests asking the senior coach.</t>
         </is>
       </c>
-      <c r="H63" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I63" s="9" t="n"/>
-      <c r="J63" s="10" t="inlineStr">
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="n"/>
+      <c r="J78" s="10" t="inlineStr">
         <is>
           <t>KNOWN ISSUE: the app says 'Your senior coach has been notified', but nothing is sent to the coach yet — judge the answer only.
 KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K63" s="11" t="inlineStr">
+      <c r="K78" s="11" t="inlineStr">
         <is>
           <t>BM</t>
         </is>
       </c>
-      <c r="L63" s="6" t="inlineStr">
+      <c r="L78" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M63" s="11" t="n">
+      <c r="M78" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N63" s="6" t="inlineStr">
+      <c r="N78" s="6" t="inlineStr">
         <is>
           <t>BM speaker</t>
         </is>
       </c>
-      <c r="O63" s="11" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="O78" s="11" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Lead sources and lead stages (中文)</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D79" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="E79" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F64" s="6" t="inlineStr">
+      <c r="F79" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "D2的客户来源有哪些？一个客户会经过哪些阶段？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="G79" s="6" t="inlineStr">
         <is>
           <t>MUST: Answers in 中文 with the 4 lead sources (listing portals, WhatsApp, walk-ins, referrals) and the 7 stages in order.
 MUST NOT: Answer in English. Add sources or stages that are not in D2's SOP.
 ALSO ACCEPTABLE: Keeps "WhatsApp" and stage names in English alongside the Chinese.</t>
         </is>
       </c>
-      <c r="H64" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I64" s="9" t="n"/>
-      <c r="J64" s="10" t="inlineStr">
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I79" s="9" t="n"/>
+      <c r="J79" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.
 KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K64" s="11" t="inlineStr">
+      <c r="K79" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L64" s="6" t="inlineStr">
+      <c r="L79" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M64" s="11" t="n">
+      <c r="M79" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N64" s="6" t="inlineStr">
+      <c r="N79" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O64" s="11" t="inlineStr">
+      <c r="O79" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B80" s="6" t="inlineStr">
         <is>
           <t>Coach / Example SOP</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>Portal lead first message and follow-up count (中文)</t>
         </is>
       </c>
-      <c r="D65" s="12" t="inlineStr">
+      <c r="D80" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr">
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="F80" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "我从房产网站收到一个询问，第一条信息应该问什么？如果对方不回复，要跟进几次？"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="G80" s="6" t="inlineStr">
         <is>
           <t>MUST: Answers in 中文: first ask own stay or rent out, not budget; follow up twice, then stop.
 MUST NOT: Answer in English. Open with a budget question.
 ALSO ACCEPTABLE: Mentions replying the same day.</t>
         </is>
       </c>
-      <c r="H65" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I65" s="9" t="n"/>
-      <c r="J65" s="10" t="inlineStr">
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="10" t="inlineStr">
         <is>
           <t>PLACEHOLDER CONTENT: this answer comes from an example SOP written by engineering. Derek to confirm or replace it before UAT; if replaced, this case is re-pointed to the real SOP.
 KNOWN ISSUE: some labels and pop-ups stay in English (for example 'Sources:' and 'No match found') — judge the answer text only.</t>
         </is>
       </c>
-      <c r="K65" s="11" t="inlineStr">
+      <c r="K80" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L65" s="6" t="inlineStr">
+      <c r="L80" s="6" t="inlineStr">
         <is>
           <t>Golden</t>
         </is>
       </c>
-      <c r="M65" s="11" t="n">
+      <c r="M80" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="N65" s="6" t="inlineStr">
+      <c r="N80" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O65" s="11" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="O80" s="11" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>Coach / Scope</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>Off-topic request (stock tip) (中文)</t>
         </is>
       </c>
-      <c r="D66" s="12" t="inlineStr">
+      <c r="D81" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="E81" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "推荐一只好的股票给我。"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G81" s="6" t="inlineStr">
         <is>
           <t>MUST: Politely declines in 中文 and steers back to D2 work.
 MUST NOT: Give a stock tip. Show a Sources row.
 ALSO ACCEPTABLE: Lists what it can help with.</t>
         </is>
       </c>
-      <c r="H66" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I66" s="9" t="n"/>
-      <c r="J66" s="10" t="inlineStr">
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="n"/>
+      <c r="J81" s="10" t="inlineStr">
         <is>
           <t>Should PASS on the current build.</t>
         </is>
       </c>
-      <c r="K66" s="11" t="inlineStr">
+      <c r="K81" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L66" s="6" t="inlineStr">
+      <c r="L81" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M66" s="11" t="n">
+      <c r="M81" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N66" s="6" t="inlineStr">
+      <c r="N81" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O66" s="11" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="O81" s="11" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>Coach / Scope</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C82" s="6" t="inlineStr">
         <is>
           <t>Paid-ads walkthrough (中文)</t>
         </is>
       </c>
-      <c r="D67" s="12" t="inlineStr">
+      <c r="D82" s="12" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="E82" s="6" t="inlineStr">
         <is>
           <t>Signed in with your tester account. Chip: Coach. New chat for every run.</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr">
+      <c r="F82" s="6" t="inlineStr">
         <is>
           <t>1. Tap New chat and set the chip to Coach.
 2. Send exactly: "请一步步教我做第一个Meta广告。"
 Then paste the full answer into the Actual / Comments column.</t>
         </is>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G82" s="6" t="inlineStr">
         <is>
           <t>MUST: Says, in 中文, that paid Meta or Google ads are not part of the D2 playbook, or that this is not in the D2 knowledge base.
 MUST NOT: Invent ad set-up steps.
 ALSO ACCEPTABLE: Suggests asking the senior coach.</t>
         </is>
       </c>
-      <c r="H67" s="8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="I67" s="9" t="n"/>
-      <c r="J67" s="10" t="inlineStr">
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="n"/>
+      <c r="J82" s="10" t="inlineStr">
         <is>
           <t>CHECK WITH DEREK: the assistant is set up to say paid ads are not part of the D2 playbook, which conflicts with the original 'first Meta ad walkthrough' goal. See Open questions.</t>
         </is>
       </c>
-      <c r="K67" s="11" t="inlineStr">
+      <c r="K82" s="11" t="inlineStr">
         <is>
           <t>中文</t>
         </is>
       </c>
-      <c r="L67" s="6" t="inlineStr">
+      <c r="L82" s="6" t="inlineStr">
         <is>
           <t>Adversarial</t>
         </is>
       </c>
-      <c r="M67" s="11" t="n">
+      <c r="M82" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="N67" s="6" t="inlineStr">
+      <c r="N82" s="6" t="inlineStr">
         <is>
           <t>中文 speaker</t>
         </is>
       </c>
-      <c r="O67" s="11" t="n"/>
+      <c r="O82" s="11" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A52:O52"/>
+  <mergeCells count="4">
+    <mergeCell ref="A46:O46"/>
+    <mergeCell ref="A67:O67"/>
     <mergeCell ref="A31:O31"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>